<commit_message>
file updates round 2
</commit_message>
<xml_diff>
--- a/InputData/elec/BPMCCS/BAU Pol Mandated Cap Const Sched.xlsx
+++ b/InputData/elec/BPMCCS/BAU Pol Mandated Cap Const Sched.xlsx
@@ -14687,13 +14687,13 @@
 </file>
 
 <file path=customXml/itemProps1.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{59FEBC86-B4BF-4815-9A76-C415776EF2B7}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{43ED1489-0F0F-460E-8DB0-F645CB7D0188}"/>
 </file>
 
 <file path=customXml/itemProps2.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{1145CB82-DA0B-43E0-AC74-05E3A110C197}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{B79B8AEF-803A-4C5A-B04E-B80AE175902F}"/>
 </file>
 
 <file path=customXml/itemProps3.xml><?xml version="1.0" encoding="utf-8"?>
-<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{BAFCB4CD-1E35-4C21-995D-D24C672E18AF}"/>
+<ds:datastoreItem xmlns:ds="http://schemas.openxmlformats.org/officeDocument/2006/customXml" ds:itemID="{5B24FF82-77E2-4C47-88CE-8E1D1040FA1D}"/>
 </file>
</xml_diff>